<commit_message>
docs(schedule): update week 1 commit progress for release engineer
</commit_message>
<xml_diff>
--- a/lich-lam-viec-commit.xlsx
+++ b/lich-lam-viec-commit.xlsx
@@ -3470,11 +3470,19 @@
       <c r="L45" s="36" t="n"/>
       <c r="M45" s="37" t="inlineStr">
         <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="N45" s="38" t="n"/>
-      <c r="O45" s="38" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N45" s="38" t="inlineStr">
+        <is>
+          <t>c52b639</t>
+        </is>
+      </c>
+      <c r="O45" s="38" t="inlineStr">
+        <is>
+          <t>Hoàn thành ngày 30/10 (Thứ 6)</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="25">
       <c r="A46" s="34" t="inlineStr">
@@ -3526,11 +3534,19 @@
       <c r="L46" s="36" t="n"/>
       <c r="M46" s="37" t="inlineStr">
         <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="N46" s="38" t="n"/>
-      <c r="O46" s="38" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N46" s="38" t="inlineStr">
+        <is>
+          <t>e7da4f3</t>
+        </is>
+      </c>
+      <c r="O46" s="38" t="inlineStr">
+        <is>
+          <t>Hoàn thành ngày 30/10 (Thứ 6)</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="23.85" customHeight="1" s="25">
       <c r="A47" s="34" t="inlineStr">

</xml_diff>

<commit_message>
docs(schedule): mark week 1 observability complete
</commit_message>
<xml_diff>
--- a/lich-lam-viec-commit.xlsx
+++ b/lich-lam-viec-commit.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hướng dẫn" sheetId="1" r:id="Rcedf76a277b84079"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lịch chi tiết" sheetId="2" r:id="Rf57d0cf6b0714a0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng hợp" sheetId="3" r:id="R1d4ac2580f054218"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hướng dẫn" sheetId="1" r:id="R1f3a626fc81e4849"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lịch chi tiết" sheetId="2" r:id="R432c4e914f1840b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng hợp" sheetId="3" r:id="R21aea104553e43d9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3800,13 +3800,13 @@
       <x:c r="K51" s="36" t="n"/>
       <x:c r="L51" s="36" t="n"/>
       <x:c r="M51" s="37" t="str">
-        <x:v>Đang làm</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="N51" s="49" t="str">
-        <x:v>3fa1b32</x:v>
+        <x:v>6b6bd5a</x:v>
       </x:c>
       <x:c r="O51" s="38" t="str">
-        <x:v>FastAPI đã được instrument, nhưng health endpoints chưa được loại trừ như nội dung kế hoạch.</x:v>
+        <x:v>Hoàn thành 25/10/2026: loại /health/live và /health/ready khỏi FastAPI tracing; 88 unit tests pass.</x:v>
       </x:c>
     </x:row>
     <x:row r="52" s="25" customFormat="1" ht="15" customHeight="1">
@@ -15842,7 +15842,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c30addf750b4d13"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4812b5cc7f744e9"/>
 </x:worksheet>
 </file>
 
@@ -16277,7 +16277,7 @@
       </x:c>
       <x:c r="B20" s="44" t="n">
         <x:f>COUNTIFS('Lịch chi tiết'!$E$7:$E$256,$A20,'Lịch chi tiết'!$B$7:$B$256,1,'Lịch chi tiết'!$M$7:$M$256,"Done")</x:f>
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C20" s="44" t="n">
         <x:f>COUNTIFS('Lịch chi tiết'!$E$7:$E$256,$A20,'Lịch chi tiết'!$B$7:$B$256,2,'Lịch chi tiết'!$M$7:$M$256,"Done")</x:f>
@@ -16297,7 +16297,7 @@
       </x:c>
       <x:c r="G20" s="45" t="n">
         <x:f>SUM(B20:F20)</x:f>
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="21" s="25" customFormat="1" ht="15" customHeight="1">
@@ -16308,7 +16308,7 @@
       </x:c>
       <x:c r="B21" s="45" t="n">
         <x:f>SUM(B16:B20)</x:f>
-        <x:v>47</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="C21" s="45" t="n">
         <x:f>SUM(C16:C20)</x:f>
@@ -16328,7 +16328,7 @@
       </x:c>
       <x:c r="G21" s="45" t="n">
         <x:f>SUM(G16:G20)</x:f>
-        <x:v>47</x:v>
+        <x:v>48</x:v>
       </x:c>
     </x:row>
     <x:row r="24" s="25" customFormat="1" ht="15" customHeight="1">
@@ -16507,7 +16507,7 @@
       </x:c>
       <x:c r="B30" s="47" t="n">
         <x:f>IF($B$2=0,0,B20/$B$2)</x:f>
-        <x:v>0.9</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C30" s="47" t="n">
         <x:f>IF($B$2=0,0,C20/$B$2)</x:f>
@@ -16527,7 +16527,7 @@
       </x:c>
       <x:c r="G30" s="48" t="n">
         <x:f>IF($B$2=0,0,G20/($B$2*5))</x:f>
-        <x:v>0.18</x:v>
+        <x:v>0.2</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -16545,6 +16545,6 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c48af6cea584705"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb51e003be7bd41ab"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(schedule): record week 2 Monday and Tuesday completion
</commit_message>
<xml_diff>
--- a/lich-lam-viec-commit.xlsx
+++ b/lich-lam-viec-commit.xlsx
@@ -5974,11 +5974,19 @@
       <c r="L87" s="41" t="n"/>
       <c r="M87" s="37" t="inlineStr">
         <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="N87" s="38" t="n"/>
-      <c r="O87" s="38" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N87" s="38" t="inlineStr">
+        <is>
+          <t>9aa9ca7</t>
+        </is>
+      </c>
+      <c r="O87" s="38" t="inlineStr">
+        <is>
+          <t>Hoàn thành sớm ngày 27/10/2026; kiểm thử script đạt. E15 chưa đo đủ 10 phút. Xem docs/evidence/loadtest/2026-10-27-week2-smoke.md</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="25">
       <c r="A88" s="39" t="inlineStr">
@@ -6034,11 +6042,19 @@
       <c r="L88" s="41" t="n"/>
       <c r="M88" s="37" t="inlineStr">
         <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="N88" s="38" t="n"/>
-      <c r="O88" s="38" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N88" s="38" t="inlineStr">
+        <is>
+          <t>e3b91c8</t>
+        </is>
+      </c>
+      <c r="O88" s="38" t="inlineStr">
+        <is>
+          <t>Hoàn thành sớm ngày 27/10/2026; kiểm thử script đạt. E15 chưa đo đủ 10 phút. Xem docs/evidence/loadtest/2026-10-27-week2-smoke.md</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="25">
       <c r="A89" s="39" t="inlineStr">
@@ -6094,11 +6110,19 @@
       <c r="L89" s="41" t="n"/>
       <c r="M89" s="37" t="inlineStr">
         <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="N89" s="38" t="n"/>
-      <c r="O89" s="38" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N89" s="38" t="inlineStr">
+        <is>
+          <t>a571ea0</t>
+        </is>
+      </c>
+      <c r="O89" s="38" t="inlineStr">
+        <is>
+          <t>Hoàn thành sớm ngày 27/10/2026; kiểm thử script đạt. E15 chưa đo đủ 10 phút. Xem docs/evidence/loadtest/2026-10-27-week2-smoke.md</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="25">
       <c r="A90" s="39" t="inlineStr">
@@ -6154,11 +6178,19 @@
       <c r="L90" s="41" t="n"/>
       <c r="M90" s="37" t="inlineStr">
         <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="N90" s="38" t="n"/>
-      <c r="O90" s="38" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N90" s="38" t="inlineStr">
+        <is>
+          <t>84f38cd</t>
+        </is>
+      </c>
+      <c r="O90" s="38" t="inlineStr">
+        <is>
+          <t>Hoàn thành sớm ngày 27/10/2026; kiểm thử script đạt. E15 chưa đo đủ 10 phút. Xem docs/evidence/loadtest/2026-10-27-week2-smoke.md</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="25">
       <c r="A91" s="39" t="inlineStr">

</xml_diff>

<commit_message>
docs(schedule): track demo load test and fault config follow-up
</commit_message>
<xml_diff>
--- a/lich-lam-viec-commit.xlsx
+++ b/lich-lam-viec-commit.xlsx
@@ -6229,11 +6229,19 @@
       </x:c>
       <x:c r="M91" s="37" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N91" s="38" t="n"/>
-      <x:c r="O91" s="38" t="n"/>
+          <x:t>Done</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N91" s="38" t="inlineStr">
+        <x:is>
+          <x:t>2e48e1b</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="O91" s="38" t="inlineStr">
+        <x:is>
+          <x:t>Hoàn thành code sớm ngày 27/10/2026. Workflow thủ công trên demo, port 80; actionlint đạt; chưa chạy GitHub Actions.</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="92" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A92" s="39" t="inlineStr">
@@ -6401,11 +6409,19 @@
       <x:c r="L94" s="41" t="n"/>
       <x:c r="M94" s="37" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N94" s="38" t="n"/>
-      <x:c r="O94" s="38" t="n"/>
+          <x:t>Done</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N94" s="38" t="inlineStr">
+        <x:is>
+          <x:t>8e4b6d7</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="O94" s="38" t="inlineStr">
+        <x:is>
+          <x:t>Hoàn thành code sớm ngày 27/10/2026. Fault config qua manifest/env; rollback về off, không migration; Compose config đạt.</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="95" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A95" s="39" t="inlineStr">
@@ -6457,11 +6473,19 @@
       <x:c r="L95" s="41" t="n"/>
       <x:c r="M95" s="37" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N95" s="38" t="n"/>
-      <x:c r="O95" s="38" t="n"/>
+          <x:t>Done</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N95" s="38" t="inlineStr">
+        <x:is>
+          <x:t>8e4b6d7</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="O95" s="38" t="inlineStr">
+        <x:is>
+          <x:t>Hoàn thành code sớm ngày 27/10/2026. Regression tests phục hồi fault config đạt; tổng 121 unit tests pass; chưa diễn tập demo.</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="96" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A96" s="39" t="inlineStr">

</xml_diff>

<commit_message>
docs(schedule): reconcile week 2 completion status
</commit_message>
<xml_diff>
--- a/lich-lam-viec-commit.xlsx
+++ b/lich-lam-viec-commit.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hướng dẫn" sheetId="1" r:id="R1f3a626fc81e4849"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lịch chi tiết" sheetId="2" r:id="R432c4e914f1840b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng hợp" sheetId="3" r:id="R21aea104553e43d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hướng dẫn" sheetId="1" r:id="Rdff0a3c469044912"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lịch chi tiết" sheetId="2" r:id="Rbe2204cae17f42ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng hợp" sheetId="3" r:id="Rdf7450b653a6495c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4167,13 +4167,15 @@
         </x:is>
       </x:c>
       <x:c r="L57" s="41" t="n"/>
-      <x:c r="M57" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N57" s="38" t="n"/>
-      <x:c r="O57" s="38" t="n"/>
+      <x:c r="M57" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N57" s="38" t="str">
+        <x:v>166e2f9</x:v>
+      </x:c>
+      <x:c r="O57" s="38" t="str">
+        <x:v>Đã merge main qua PR #26; runbook demo host đã có.</x:v>
+      </x:c>
     </x:row>
     <x:row r="58" s="25" customFormat="1" ht="23.850000381469727" customHeight="1">
       <x:c r="A58" s="39" t="inlineStr">
@@ -4227,13 +4229,15 @@
         </x:is>
       </x:c>
       <x:c r="L58" s="41" t="n"/>
-      <x:c r="M58" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N58" s="38" t="n"/>
-      <x:c r="O58" s="38" t="n"/>
+      <x:c r="M58" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N58" s="38" t="str">
+        <x:v>848857c</x:v>
+      </x:c>
+      <x:c r="O58" s="38" t="str">
+        <x:v>Đã merge main qua PR #26; bootstrap Docker/state dir đã có.</x:v>
+      </x:c>
     </x:row>
     <x:row r="59" s="25" customFormat="1" ht="23.850000381469727" customHeight="1">
       <x:c r="A59" s="39" t="inlineStr">
@@ -4291,13 +4295,15 @@
           <x:t xml:space="preserve">Runner đã online</x:t>
         </x:is>
       </x:c>
-      <x:c r="M59" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N59" s="38" t="n"/>
-      <x:c r="O59" s="38" t="n"/>
+      <x:c r="M59" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N59" s="38" t="str">
+        <x:v>e84b0af</x:v>
+      </x:c>
+      <x:c r="O59" s="38" t="str">
+        <x:v>Workflow code đã merge; runner demo thật vẫn cần admin đăng ký.</x:v>
+      </x:c>
     </x:row>
     <x:row r="60" s="25" customFormat="1" ht="23.850000381469727" customHeight="1">
       <x:c r="A60" s="39" t="inlineStr">
@@ -4351,13 +4357,15 @@
         </x:is>
       </x:c>
       <x:c r="L60" s="41" t="n"/>
-      <x:c r="M60" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N60" s="38" t="n"/>
-      <x:c r="O60" s="38" t="n"/>
+      <x:c r="M60" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N60" s="38" t="str">
+        <x:v>69a37b1</x:v>
+      </x:c>
+      <x:c r="O60" s="38" t="str">
+        <x:v>Đã merge main qua PR #26; có workflow_run sau release.</x:v>
+      </x:c>
     </x:row>
     <x:row r="61" s="25" customFormat="1" ht="23.850000381469727" customHeight="1">
       <x:c r="A61" s="39" t="inlineStr">
@@ -4411,13 +4419,15 @@
         </x:is>
       </x:c>
       <x:c r="L61" s="41" t="n"/>
-      <x:c r="M61" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N61" s="38" t="n"/>
-      <x:c r="O61" s="38" t="n"/>
+      <x:c r="M61" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N61" s="38" t="str">
+        <x:v>6510809</x:v>
+      </x:c>
+      <x:c r="O61" s="38" t="str">
+        <x:v>Đã merge main qua PR #26; artifact log/manifests đã cấu hình.</x:v>
+      </x:c>
     </x:row>
     <x:row r="62" s="25" customFormat="1" ht="23.850000381469727" customHeight="1">
       <x:c r="A62" s="39" t="inlineStr">
@@ -4475,13 +4485,15 @@
           <x:t xml:space="preserve">Việt Anh: state dir configurable (T1)</x:t>
         </x:is>
       </x:c>
-      <x:c r="M62" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N62" s="38" t="n"/>
-      <x:c r="O62" s="38" t="n"/>
+      <x:c r="M62" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N62" s="38" t="str">
+        <x:v>16bb17c</x:v>
+      </x:c>
+      <x:c r="O62" s="38" t="str">
+        <x:v>Đã merge main qua PR #26; rollback dùng self-hosted demo runner.</x:v>
+      </x:c>
     </x:row>
     <x:row r="63" s="25" customFormat="1" ht="23.850000381469727" customHeight="1">
       <x:c r="A63" s="39" t="inlineStr">
@@ -4535,13 +4547,15 @@
         </x:is>
       </x:c>
       <x:c r="L63" s="41" t="n"/>
-      <x:c r="M63" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N63" s="38" t="n"/>
-      <x:c r="O63" s="38" t="n"/>
+      <x:c r="M63" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N63" s="38" t="str">
+        <x:v>2e4c14b</x:v>
+      </x:c>
+      <x:c r="O63" s="38" t="str">
+        <x:v>Đã merge main qua PR #26; deploy/rollback dùng group deploy-demo.</x:v>
+      </x:c>
     </x:row>
     <x:row r="64" s="25" customFormat="1" ht="23.850000381469727" customHeight="1">
       <x:c r="A64" s="39" t="inlineStr">
@@ -4595,13 +4609,15 @@
         </x:is>
       </x:c>
       <x:c r="L64" s="41" t="n"/>
-      <x:c r="M64" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N64" s="38" t="n"/>
-      <x:c r="O64" s="38" t="n"/>
+      <x:c r="M64" s="37" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="N64" s="38" t="str">
+        <x:v>7c73e26</x:v>
+      </x:c>
+      <x:c r="O64" s="38" t="str">
+        <x:v>Workflow đã gắn environment demo; required reviewer còn cần admin xác nhận.</x:v>
+      </x:c>
     </x:row>
     <x:row r="65" s="25" customFormat="1" ht="23.850000381469727" customHeight="1">
       <x:c r="A65" s="39" t="inlineStr">
@@ -4659,13 +4675,15 @@
           <x:t xml:space="preserve">Cường: Dockerfile frontend (T2)</x:t>
         </x:is>
       </x:c>
-      <x:c r="M65" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N65" s="38" t="n"/>
-      <x:c r="O65" s="38" t="n"/>
+      <x:c r="M65" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N65" s="38" t="str">
+        <x:v>6919bd0</x:v>
+      </x:c>
+      <x:c r="O65" s="38" t="str">
+        <x:v>Đã merge main qua PR #26; chỉ Nginx public, backend/DB nội bộ.</x:v>
+      </x:c>
     </x:row>
     <x:row r="66" s="25" customFormat="1" ht="23.850000381469727" customHeight="1">
       <x:c r="A66" s="39" t="inlineStr">
@@ -4719,13 +4737,15 @@
         </x:is>
       </x:c>
       <x:c r="L66" s="41" t="n"/>
-      <x:c r="M66" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N66" s="38" t="n"/>
-      <x:c r="O66" s="38" t="n"/>
+      <x:c r="M66" s="37" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="N66" s="38" t="str">
+        <x:v>58a5fbc</x:v>
+      </x:c>
+      <x:c r="O66" s="38" t="str">
+        <x:v>Có rehearsal local; chưa có GitHub deploy run trên demo để chốt E08.</x:v>
+      </x:c>
     </x:row>
     <x:row r="67" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A67" s="39" t="inlineStr">
@@ -4779,13 +4799,15 @@
         </x:is>
       </x:c>
       <x:c r="L67" s="41" t="n"/>
-      <x:c r="M67" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N67" s="38" t="n"/>
-      <x:c r="O67" s="38" t="n"/>
+      <x:c r="M67" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N67" s="38" t="str">
+        <x:v>3fa1b32</x:v>
+      </x:c>
+      <x:c r="O67" s="38" t="str">
+        <x:v>JSON request logging đã có và unit tests đạt.</x:v>
+      </x:c>
     </x:row>
     <x:row r="68" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A68" s="39" t="inlineStr">
@@ -4839,13 +4861,15 @@
         </x:is>
       </x:c>
       <x:c r="L68" s="41" t="n"/>
-      <x:c r="M68" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N68" s="38" t="n"/>
-      <x:c r="O68" s="38" t="n"/>
+      <x:c r="M68" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N68" s="38" t="str">
+        <x:v>3fa1b32</x:v>
+      </x:c>
+      <x:c r="O68" s="38" t="str">
+        <x:v>Middleware ghi method/route/status/duration đã có.</x:v>
+      </x:c>
     </x:row>
     <x:row r="69" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A69" s="39" t="inlineStr">
@@ -4899,13 +4923,15 @@
         </x:is>
       </x:c>
       <x:c r="L69" s="41" t="n"/>
-      <x:c r="M69" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N69" s="38" t="n"/>
-      <x:c r="O69" s="38" t="n"/>
+      <x:c r="M69" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N69" s="38" t="str">
+        <x:v>3fa1b32</x:v>
+      </x:c>
+      <x:c r="O69" s="38" t="str">
+        <x:v>Test xác nhận log không chứa body/tên khách.</x:v>
+      </x:c>
     </x:row>
     <x:row r="70" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A70" s="39" t="inlineStr">
@@ -4959,13 +4985,15 @@
         </x:is>
       </x:c>
       <x:c r="L70" s="41" t="n"/>
-      <x:c r="M70" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N70" s="38" t="n"/>
-      <x:c r="O70" s="38" t="n"/>
+      <x:c r="M70" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N70" s="38" t="str">
+        <x:v>7ca61e0</x:v>
+      </x:c>
+      <x:c r="O70" s="38" t="str">
+        <x:v>/api/version trả environment và fault_active; unit tests đạt.</x:v>
+      </x:c>
     </x:row>
     <x:row r="71" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A71" s="39" t="inlineStr">
@@ -5019,13 +5047,15 @@
         </x:is>
       </x:c>
       <x:c r="L71" s="41" t="n"/>
-      <x:c r="M71" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N71" s="38" t="n"/>
-      <x:c r="O71" s="38" t="n"/>
+      <x:c r="M71" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N71" s="38" t="str">
+        <x:v>3fa1b32</x:v>
+      </x:c>
+      <x:c r="O71" s="38" t="str">
+        <x:v>Route template cố định được dùng cho log/telemetry labels.</x:v>
+      </x:c>
     </x:row>
     <x:row r="72" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A72" s="39" t="inlineStr">
@@ -5079,13 +5109,15 @@
         </x:is>
       </x:c>
       <x:c r="L72" s="41" t="n"/>
-      <x:c r="M72" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N72" s="38" t="n"/>
-      <x:c r="O72" s="38" t="n"/>
+      <x:c r="M72" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N72" s="38" t="str">
+        <x:v>7ca61e0</x:v>
+      </x:c>
+      <x:c r="O72" s="38" t="str">
+        <x:v>Readiness trả database_check_ms cho ready/unavailable.</x:v>
+      </x:c>
     </x:row>
     <x:row r="73" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A73" s="39" t="inlineStr">
@@ -5139,13 +5171,15 @@
         </x:is>
       </x:c>
       <x:c r="L73" s="41" t="n"/>
-      <x:c r="M73" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N73" s="38" t="n"/>
-      <x:c r="O73" s="38" t="n"/>
+      <x:c r="M73" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N73" s="38" t="str">
+        <x:v>7ca61e0</x:v>
+      </x:c>
+      <x:c r="O73" s="38" t="str">
+        <x:v>Test DB chậm xác nhận 503 trong timeout hữu hạn.</x:v>
+      </x:c>
     </x:row>
     <x:row r="74" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A74" s="39" t="inlineStr">
@@ -5199,13 +5233,15 @@
         </x:is>
       </x:c>
       <x:c r="L74" s="41" t="n"/>
-      <x:c r="M74" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N74" s="38" t="n"/>
-      <x:c r="O74" s="38" t="n"/>
+      <x:c r="M74" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N74" s="38" t="str">
+        <x:v>7ca61e0</x:v>
+      </x:c>
+      <x:c r="O74" s="38" t="str">
+        <x:v>Test limit 0/101 và offset âm trả 422.</x:v>
+      </x:c>
     </x:row>
     <x:row r="75" s="25" customFormat="1" ht="23.850000381469727" customHeight="1">
       <x:c r="A75" s="39" t="inlineStr">
@@ -5259,13 +5295,15 @@
         </x:is>
       </x:c>
       <x:c r="L75" s="41" t="n"/>
-      <x:c r="M75" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N75" s="38" t="n"/>
-      <x:c r="O75" s="38" t="n"/>
+      <x:c r="M75" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N75" s="38" t="str">
+        <x:v>3fa1b32</x:v>
+      </x:c>
+      <x:c r="O75" s="38" t="str">
+        <x:v>Booking create/cancel có span nghiệp vụ riêng.</x:v>
+      </x:c>
     </x:row>
     <x:row r="76" s="25" customFormat="1" ht="23.850000381469727" customHeight="1">
       <x:c r="A76" s="39" t="inlineStr">
@@ -5319,13 +5357,15 @@
         </x:is>
       </x:c>
       <x:c r="L76" s="41" t="n"/>
-      <x:c r="M76" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N76" s="38" t="n"/>
-      <x:c r="O76" s="38" t="n"/>
+      <x:c r="M76" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N76" s="38" t="str">
+        <x:v>3fa1b32</x:v>
+      </x:c>
+      <x:c r="O76" s="38" t="str">
+        <x:v>Module view đã mô tả telemetry và fault injection.</x:v>
+      </x:c>
     </x:row>
     <x:row r="77" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A77" s="39" t="inlineStr">
@@ -5379,13 +5419,15 @@
         </x:is>
       </x:c>
       <x:c r="L77" s="41" t="n"/>
-      <x:c r="M77" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N77" s="38" t="n"/>
-      <x:c r="O77" s="38" t="n"/>
+      <x:c r="M77" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N77" s="38" t="str">
+        <x:v>daecbc6</x:v>
+      </x:c>
+      <x:c r="O77" s="38" t="str">
+        <x:v>Hoàn thành gộp trong TASK-003; evidence frontend 25/10.</x:v>
+      </x:c>
     </x:row>
     <x:row r="78" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A78" s="39" t="inlineStr">
@@ -5439,13 +5481,15 @@
         </x:is>
       </x:c>
       <x:c r="L78" s="41" t="n"/>
-      <x:c r="M78" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N78" s="38" t="n"/>
-      <x:c r="O78" s="38" t="n"/>
+      <x:c r="M78" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N78" s="38" t="str">
+        <x:v>daecbc6</x:v>
+      </x:c>
+      <x:c r="O78" s="38" t="str">
+        <x:v>Hoàn thành gộp trong TASK-003; 409 không báo thành công.</x:v>
+      </x:c>
     </x:row>
     <x:row r="79" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A79" s="39" t="inlineStr">
@@ -5495,13 +5539,15 @@
       </x:c>
       <x:c r="K79" s="41" t="n"/>
       <x:c r="L79" s="41" t="n"/>
-      <x:c r="M79" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N79" s="38" t="n"/>
-      <x:c r="O79" s="38" t="n"/>
+      <x:c r="M79" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N79" s="38" t="str">
+        <x:v>daecbc6</x:v>
+      </x:c>
+      <x:c r="O79" s="38" t="str">
+        <x:v>Hoàn thành gộp trong TASK-003; component tests đạt.</x:v>
+      </x:c>
     </x:row>
     <x:row r="80" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A80" s="39" t="inlineStr">
@@ -5551,13 +5597,15 @@
       </x:c>
       <x:c r="K80" s="41" t="n"/>
       <x:c r="L80" s="41" t="n"/>
-      <x:c r="M80" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N80" s="38" t="n"/>
-      <x:c r="O80" s="38" t="n"/>
+      <x:c r="M80" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N80" s="38" t="str">
+        <x:v>daecbc6</x:v>
+      </x:c>
+      <x:c r="O80" s="38" t="str">
+        <x:v>Hoàn thành gộp trong TASK-003; pagination đã có.</x:v>
+      </x:c>
     </x:row>
     <x:row r="81" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A81" s="39" t="inlineStr">
@@ -5611,13 +5659,15 @@
         </x:is>
       </x:c>
       <x:c r="L81" s="41" t="n"/>
-      <x:c r="M81" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N81" s="38" t="n"/>
-      <x:c r="O81" s="38" t="n"/>
+      <x:c r="M81" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N81" s="38" t="str">
+        <x:v>daecbc6</x:v>
+      </x:c>
+      <x:c r="O81" s="38" t="str">
+        <x:v>Hoàn thành gộp trong TASK-003; cancel có xác nhận.</x:v>
+      </x:c>
     </x:row>
     <x:row r="82" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A82" s="39" t="inlineStr">
@@ -5667,13 +5717,15 @@
       </x:c>
       <x:c r="K82" s="41" t="n"/>
       <x:c r="L82" s="41" t="n"/>
-      <x:c r="M82" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N82" s="38" t="n"/>
-      <x:c r="O82" s="38" t="n"/>
+      <x:c r="M82" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N82" s="38" t="str">
+        <x:v>daecbc6</x:v>
+      </x:c>
+      <x:c r="O82" s="38" t="str">
+        <x:v>Hoàn thành gộp trong TASK-003; cancel tests đạt.</x:v>
+      </x:c>
     </x:row>
     <x:row r="83" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A83" s="39" t="inlineStr">
@@ -5727,13 +5779,15 @@
         </x:is>
       </x:c>
       <x:c r="L83" s="41" t="n"/>
-      <x:c r="M83" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N83" s="38" t="n"/>
-      <x:c r="O83" s="38" t="n"/>
+      <x:c r="M83" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N83" s="38" t="str">
+        <x:v>daecbc6</x:v>
+      </x:c>
+      <x:c r="O83" s="38" t="str">
+        <x:v>Hoàn thành gộp trong TASK-003; footer release/commit đã có.</x:v>
+      </x:c>
     </x:row>
     <x:row r="84" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A84" s="39" t="inlineStr">
@@ -5783,13 +5837,15 @@
       </x:c>
       <x:c r="K84" s="41" t="n"/>
       <x:c r="L84" s="41" t="n"/>
-      <x:c r="M84" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N84" s="38" t="n"/>
-      <x:c r="O84" s="38" t="n"/>
+      <x:c r="M84" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N84" s="38" t="str">
+        <x:v>daecbc6</x:v>
+      </x:c>
+      <x:c r="O84" s="38" t="str">
+        <x:v>Hoàn thành gộp trong TASK-003; layout responsive đã có.</x:v>
+      </x:c>
     </x:row>
     <x:row r="85" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A85" s="39" t="inlineStr">
@@ -5843,13 +5899,15 @@
         </x:is>
       </x:c>
       <x:c r="L85" s="41" t="n"/>
-      <x:c r="M85" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N85" s="38" t="n"/>
-      <x:c r="O85" s="38" t="n"/>
+      <x:c r="M85" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N85" s="38" t="str">
+        <x:v>daecbc6</x:v>
+      </x:c>
+      <x:c r="O85" s="38" t="str">
+        <x:v>Hoàn thành gộp trong TASK-003; frontend Dockerfile multi-stage.</x:v>
+      </x:c>
     </x:row>
     <x:row r="86" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A86" s="39" t="inlineStr">
@@ -5899,13 +5957,15 @@
       </x:c>
       <x:c r="K86" s="41" t="n"/>
       <x:c r="L86" s="41" t="n"/>
-      <x:c r="M86" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N86" s="38" t="n"/>
-      <x:c r="O86" s="38" t="n"/>
+      <x:c r="M86" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N86" s="38" t="str">
+        <x:v>daecbc6</x:v>
+      </x:c>
+      <x:c r="O86" s="38" t="str">
+        <x:v>Hoàn thành gộp trong TASK-003; Nginx proxy /api và /health.</x:v>
+      </x:c>
     </x:row>
     <x:row r="87" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A87" s="39" t="inlineStr">
@@ -5955,20 +6015,14 @@
       </x:c>
       <x:c r="K87" s="41" t="n"/>
       <x:c r="L87" s="41" t="n"/>
-      <x:c r="M87" s="37" t="inlineStr">
-        <x:is>
-          <x:t>Done</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N87" s="38" t="inlineStr">
-        <x:is>
-          <x:t>9aa9ca7</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O87" s="38" t="inlineStr">
-        <x:is>
-          <x:t>Hoàn thành sớm ngày 27/10/2026; kiểm thử script đạt. E15 chưa đo đủ 10 phút. Xem docs/evidence/loadtest/2026-10-27-week2-smoke.md</x:t>
-        </x:is>
+      <x:c r="M87" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N87" s="38" t="str">
+        <x:v>9aa9ca7</x:v>
+      </x:c>
+      <x:c r="O87" s="38" t="str">
+        <x:v>Hoàn thành sớm ngày 27/10/2026; kiểm thử script đạt. E15 chưa đo đủ 10 phút. Xem docs/evidence/loadtest/2026-10-27-week2-smoke.md</x:v>
       </x:c>
     </x:row>
     <x:row r="88" s="25" customFormat="1" ht="15" customHeight="1">
@@ -6023,20 +6077,14 @@
         </x:is>
       </x:c>
       <x:c r="L88" s="41" t="n"/>
-      <x:c r="M88" s="37" t="inlineStr">
-        <x:is>
-          <x:t>Done</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N88" s="38" t="inlineStr">
-        <x:is>
-          <x:t>e3b91c8</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O88" s="38" t="inlineStr">
-        <x:is>
-          <x:t>Hoàn thành sớm ngày 27/10/2026; kiểm thử script đạt. E15 chưa đo đủ 10 phút. Xem docs/evidence/loadtest/2026-10-27-week2-smoke.md</x:t>
-        </x:is>
+      <x:c r="M88" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N88" s="38" t="str">
+        <x:v>e3b91c8</x:v>
+      </x:c>
+      <x:c r="O88" s="38" t="str">
+        <x:v>Hoàn thành sớm ngày 27/10/2026; kiểm thử script đạt. E15 chưa đo đủ 10 phút. Xem docs/evidence/loadtest/2026-10-27-week2-smoke.md</x:v>
       </x:c>
     </x:row>
     <x:row r="89" s="25" customFormat="1" ht="15" customHeight="1">
@@ -6091,20 +6139,14 @@
         </x:is>
       </x:c>
       <x:c r="L89" s="41" t="n"/>
-      <x:c r="M89" s="37" t="inlineStr">
-        <x:is>
-          <x:t>Done</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N89" s="38" t="inlineStr">
-        <x:is>
-          <x:t>a571ea0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O89" s="38" t="inlineStr">
-        <x:is>
-          <x:t>Hoàn thành sớm ngày 27/10/2026; kiểm thử script đạt. E15 chưa đo đủ 10 phút. Xem docs/evidence/loadtest/2026-10-27-week2-smoke.md</x:t>
-        </x:is>
+      <x:c r="M89" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N89" s="38" t="str">
+        <x:v>a571ea0</x:v>
+      </x:c>
+      <x:c r="O89" s="38" t="str">
+        <x:v>Hoàn thành sớm ngày 27/10/2026; kiểm thử script đạt. E15 chưa đo đủ 10 phút. Xem docs/evidence/loadtest/2026-10-27-week2-smoke.md</x:v>
       </x:c>
     </x:row>
     <x:row r="90" s="25" customFormat="1" ht="15" customHeight="1">
@@ -6159,20 +6201,14 @@
         </x:is>
       </x:c>
       <x:c r="L90" s="41" t="n"/>
-      <x:c r="M90" s="37" t="inlineStr">
-        <x:is>
-          <x:t>Done</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N90" s="38" t="inlineStr">
-        <x:is>
-          <x:t>84f38cd</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O90" s="38" t="inlineStr">
-        <x:is>
-          <x:t>Hoàn thành sớm ngày 27/10/2026; kiểm thử script đạt. E15 chưa đo đủ 10 phút. Xem docs/evidence/loadtest/2026-10-27-week2-smoke.md</x:t>
-        </x:is>
+      <x:c r="M90" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N90" s="38" t="str">
+        <x:v>84f38cd</x:v>
+      </x:c>
+      <x:c r="O90" s="38" t="str">
+        <x:v>Hoàn thành sớm ngày 27/10/2026; kiểm thử script đạt. E15 chưa đo đủ 10 phút. Xem docs/evidence/loadtest/2026-10-27-week2-smoke.md</x:v>
       </x:c>
     </x:row>
     <x:row r="91" s="25" customFormat="1" ht="15" customHeight="1">
@@ -6227,20 +6263,14 @@
           <x:t xml:space="preserve">Hoàng Anh: runner (T2)</x:t>
         </x:is>
       </x:c>
-      <x:c r="M91" s="37" t="inlineStr">
-        <x:is>
-          <x:t>Done</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N91" s="38" t="inlineStr">
-        <x:is>
-          <x:t>2e48e1b</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O91" s="38" t="inlineStr">
-        <x:is>
-          <x:t>Hoàn thành code sớm ngày 27/10/2026. Workflow thủ công trên demo, port 80; actionlint đạt; chưa chạy GitHub Actions.</x:t>
-        </x:is>
+      <x:c r="M91" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N91" s="38" t="str">
+        <x:v>2e48e1b</x:v>
+      </x:c>
+      <x:c r="O91" s="38" t="str">
+        <x:v>Hoàn thành code sớm ngày 27/10/2026. Workflow thủ công trên demo, port 80; actionlint đạt; chưa chạy GitHub Actions.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" s="25" customFormat="1" ht="15" customHeight="1">
@@ -6291,13 +6321,15 @@
       </x:c>
       <x:c r="K92" s="41" t="n"/>
       <x:c r="L92" s="41" t="n"/>
-      <x:c r="M92" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N92" s="38" t="n"/>
-      <x:c r="O92" s="38" t="n"/>
+      <x:c r="M92" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N92" s="38" t="str">
+        <x:v>3df685d</x:v>
+      </x:c>
+      <x:c r="O92" s="38" t="str">
+        <x:v>Smoke test đối chiếu release và commit_sha với manifest.</x:v>
+      </x:c>
     </x:row>
     <x:row r="93" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A93" s="39" t="inlineStr">
@@ -6347,13 +6379,15 @@
       </x:c>
       <x:c r="K93" s="41" t="n"/>
       <x:c r="L93" s="41" t="n"/>
-      <x:c r="M93" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N93" s="38" t="n"/>
-      <x:c r="O93" s="38" t="n"/>
+      <x:c r="M93" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N93" s="38" t="str">
+        <x:v>3df685d</x:v>
+      </x:c>
+      <x:c r="O93" s="38" t="str">
+        <x:v>Unit tests cover version match và mismatch.</x:v>
+      </x:c>
     </x:row>
     <x:row r="94" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A94" s="39" t="inlineStr">
@@ -6407,20 +6441,14 @@
         </x:is>
       </x:c>
       <x:c r="L94" s="41" t="n"/>
-      <x:c r="M94" s="37" t="inlineStr">
-        <x:is>
-          <x:t>Done</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N94" s="38" t="inlineStr">
-        <x:is>
-          <x:t>8e4b6d7</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O94" s="38" t="inlineStr">
-        <x:is>
-          <x:t>Hoàn thành code sớm ngày 27/10/2026. Fault config qua manifest/env; rollback về off, không migration; Compose config đạt.</x:t>
-        </x:is>
+      <x:c r="M94" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N94" s="38" t="str">
+        <x:v>8e4b6d7</x:v>
+      </x:c>
+      <x:c r="O94" s="38" t="str">
+        <x:v>Hoàn thành code sớm ngày 27/10/2026. Fault config qua manifest/env; rollback về off, không migration; Compose config đạt.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" s="25" customFormat="1" ht="15" customHeight="1">
@@ -6471,20 +6499,14 @@
       </x:c>
       <x:c r="K95" s="41" t="n"/>
       <x:c r="L95" s="41" t="n"/>
-      <x:c r="M95" s="37" t="inlineStr">
-        <x:is>
-          <x:t>Done</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N95" s="38" t="inlineStr">
-        <x:is>
-          <x:t>8e4b6d7</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O95" s="38" t="inlineStr">
-        <x:is>
-          <x:t>Hoàn thành code sớm ngày 27/10/2026. Regression tests phục hồi fault config đạt; tổng 121 unit tests pass; chưa diễn tập demo.</x:t>
-        </x:is>
+      <x:c r="M95" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N95" s="38" t="str">
+        <x:v>8e4b6d7</x:v>
+      </x:c>
+      <x:c r="O95" s="38" t="str">
+        <x:v>Hoàn thành code sớm ngày 27/10/2026. Regression tests phục hồi fault config đạt; tổng 121 unit tests pass; chưa diễn tập demo.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" s="25" customFormat="1" ht="15" customHeight="1">
@@ -6535,13 +6557,15 @@
       </x:c>
       <x:c r="K96" s="41" t="n"/>
       <x:c r="L96" s="41" t="n"/>
-      <x:c r="M96" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N96" s="38" t="n"/>
-      <x:c r="O96" s="38" t="n"/>
+      <x:c r="M96" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N96" s="38" t="str">
+        <x:v>816c3b6</x:v>
+      </x:c>
+      <x:c r="O96" s="38" t="str">
+        <x:v>Release process đã có quy trình rollback và smoke verification.</x:v>
+      </x:c>
     </x:row>
     <x:row r="97" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A97" s="39" t="inlineStr">
@@ -6591,13 +6615,15 @@
       </x:c>
       <x:c r="K97" s="41" t="n"/>
       <x:c r="L97" s="41" t="n"/>
-      <x:c r="M97" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N97" s="38" t="n"/>
-      <x:c r="O97" s="38" t="n"/>
+      <x:c r="M97" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N97" s="38" t="str">
+        <x:v>3fa1b32</x:v>
+      </x:c>
+      <x:c r="O97" s="38" t="str">
+        <x:v>OTLP metric exporter đã có trong telemetry runtime.</x:v>
+      </x:c>
     </x:row>
     <x:row r="98" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A98" s="39" t="inlineStr">
@@ -6647,13 +6673,15 @@
       </x:c>
       <x:c r="K98" s="41" t="n"/>
       <x:c r="L98" s="41" t="n"/>
-      <x:c r="M98" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N98" s="38" t="n"/>
-      <x:c r="O98" s="38" t="n"/>
+      <x:c r="M98" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N98" s="38" t="str">
+        <x:v>072ba36</x:v>
+      </x:c>
+      <x:c r="O98" s="38" t="str">
+        <x:v>HTTP duration có explicit buckets cho stable/legacy metrics.</x:v>
+      </x:c>
     </x:row>
     <x:row r="99" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A99" s="39" t="inlineStr">
@@ -6703,13 +6731,15 @@
       </x:c>
       <x:c r="K99" s="41" t="n"/>
       <x:c r="L99" s="41" t="n"/>
-      <x:c r="M99" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N99" s="38" t="n"/>
-      <x:c r="O99" s="38" t="n"/>
+      <x:c r="M99" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N99" s="38" t="str">
+        <x:v>3fa1b32</x:v>
+      </x:c>
+      <x:c r="O99" s="38" t="str">
+        <x:v>Tests xác nhận route labels dùng template, không UUID.</x:v>
+      </x:c>
     </x:row>
     <x:row r="100" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A100" s="39" t="inlineStr">
@@ -6759,13 +6789,15 @@
       </x:c>
       <x:c r="K100" s="41" t="n"/>
       <x:c r="L100" s="41" t="n"/>
-      <x:c r="M100" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N100" s="38" t="n"/>
-      <x:c r="O100" s="38" t="n"/>
+      <x:c r="M100" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N100" s="38" t="str">
+        <x:v>3fa1b32</x:v>
+      </x:c>
+      <x:c r="O100" s="38" t="str">
+        <x:v>OTLP logs bridge và bounded batch processor đã có.</x:v>
+      </x:c>
     </x:row>
     <x:row r="101" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A101" s="39" t="inlineStr">
@@ -6819,13 +6851,15 @@
         </x:is>
       </x:c>
       <x:c r="L101" s="41" t="n"/>
-      <x:c r="M101" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N101" s="38" t="n"/>
-      <x:c r="O101" s="38" t="n"/>
+      <x:c r="M101" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N101" s="38" t="str">
+        <x:v>3fa1b32</x:v>
+      </x:c>
+      <x:c r="O101" s="38" t="str">
+        <x:v>Test booking không bị block khi Collector lỗi; có E10 local.</x:v>
+      </x:c>
     </x:row>
     <x:row r="102" s="25" customFormat="1" ht="23.850000381469727" customHeight="1">
       <x:c r="A102" s="39" t="inlineStr">
@@ -6875,13 +6909,15 @@
       </x:c>
       <x:c r="K102" s="41" t="n"/>
       <x:c r="L102" s="41" t="n"/>
-      <x:c r="M102" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N102" s="38" t="n"/>
-      <x:c r="O102" s="38" t="n"/>
+      <x:c r="M102" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N102" s="38" t="str">
+        <x:v>3fa1b32</x:v>
+      </x:c>
+      <x:c r="O102" s="38" t="str">
+        <x:v>Exporter timeout, queue và batch size cấu hình được.</x:v>
+      </x:c>
     </x:row>
     <x:row r="103" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A103" s="39" t="inlineStr">
@@ -6931,13 +6967,15 @@
       </x:c>
       <x:c r="K103" s="41" t="n"/>
       <x:c r="L103" s="41" t="n"/>
-      <x:c r="M103" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N103" s="38" t="n"/>
-      <x:c r="O103" s="38" t="n"/>
+      <x:c r="M103" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N103" s="38" t="str">
+        <x:v>3fa1b32</x:v>
+      </x:c>
+      <x:c r="O103" s="38" t="str">
+        <x:v>Test outage xác nhận request path không chờ exporter.</x:v>
+      </x:c>
     </x:row>
     <x:row r="104" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A104" s="39" t="inlineStr">
@@ -6991,13 +7029,15 @@
         </x:is>
       </x:c>
       <x:c r="L104" s="41" t="n"/>
-      <x:c r="M104" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N104" s="38" t="n"/>
-      <x:c r="O104" s="38" t="n"/>
+      <x:c r="M104" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N104" s="38" t="str">
+        <x:v>072ba36</x:v>
+      </x:c>
+      <x:c r="O104" s="38" t="str">
+        <x:v>SDK bật TraceBasedExemplarFilter; Grafana/Tempo correlation đã có.</x:v>
+      </x:c>
     </x:row>
     <x:row r="105" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A105" s="39" t="inlineStr">
@@ -7047,13 +7087,15 @@
       </x:c>
       <x:c r="K105" s="41" t="n"/>
       <x:c r="L105" s="41" t="n"/>
-      <x:c r="M105" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N105" s="38" t="n"/>
-      <x:c r="O105" s="38" t="n"/>
+      <x:c r="M105" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N105" s="38" t="str">
+        <x:v>3fa1b32</x:v>
+      </x:c>
+      <x:c r="O105" s="38" t="str">
+        <x:v>backend README đã mô tả telemetry environment variables.</x:v>
+      </x:c>
     </x:row>
     <x:row r="106" s="25" customFormat="1" ht="15" customHeight="1">
       <x:c r="A106" s="39" t="inlineStr">
@@ -7103,13 +7145,15 @@
       </x:c>
       <x:c r="K106" s="41" t="n"/>
       <x:c r="L106" s="41" t="n"/>
-      <x:c r="M106" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Todo</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N106" s="38" t="n"/>
-      <x:c r="O106" s="38" t="n"/>
+      <x:c r="M106" s="37" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N106" s="38" t="str">
+        <x:v>a80423e</x:v>
+      </x:c>
+      <x:c r="O106" s="38" t="str">
+        <x:v>Đã lưu E10 local Collector outage drill; demo chung vẫn còn.</x:v>
+      </x:c>
     </x:row>
     <x:row r="107" s="25" customFormat="1" ht="23.850000381469727" customHeight="1">
       <x:c r="A107" s="34" t="inlineStr">
@@ -15898,7 +15942,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4812b5cc7f744e9"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81e45ced4afc4bed"/>
 </x:worksheet>
 </file>
 
@@ -16213,7 +16257,7 @@
       </x:c>
       <x:c r="C16" s="44" t="n">
         <x:f>COUNTIFS('Lịch chi tiết'!$E$7:$E$256,$A16,'Lịch chi tiết'!$B$7:$B$256,2,'Lịch chi tiết'!$M$7:$M$256,"Done")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D16" s="44" t="n">
         <x:f>COUNTIFS('Lịch chi tiết'!$E$7:$E$256,$A16,'Lịch chi tiết'!$B$7:$B$256,3,'Lịch chi tiết'!$M$7:$M$256,"Done")</x:f>
@@ -16229,7 +16273,7 @@
       </x:c>
       <x:c r="G16" s="45" t="n">
         <x:f>SUM(B16:F16)</x:f>
-        <x:v>10</x:v>
+        <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="17" s="25" customFormat="1" ht="15" customHeight="1">
@@ -16244,7 +16288,7 @@
       </x:c>
       <x:c r="C17" s="44" t="n">
         <x:f>COUNTIFS('Lịch chi tiết'!$E$7:$E$256,$A17,'Lịch chi tiết'!$B$7:$B$256,2,'Lịch chi tiết'!$M$7:$M$256,"Done")</x:f>
-        <x:v>0</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D17" s="44" t="n">
         <x:f>COUNTIFS('Lịch chi tiết'!$E$7:$E$256,$A17,'Lịch chi tiết'!$B$7:$B$256,3,'Lịch chi tiết'!$M$7:$M$256,"Done")</x:f>
@@ -16260,7 +16304,7 @@
       </x:c>
       <x:c r="G17" s="45" t="n">
         <x:f>SUM(B17:F17)</x:f>
-        <x:v>8</x:v>
+        <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="18" s="25" customFormat="1" ht="15" customHeight="1">
@@ -16275,7 +16319,7 @@
       </x:c>
       <x:c r="C18" s="44" t="n">
         <x:f>COUNTIFS('Lịch chi tiết'!$E$7:$E$256,$A18,'Lịch chi tiết'!$B$7:$B$256,2,'Lịch chi tiết'!$M$7:$M$256,"Done")</x:f>
-        <x:v>0</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D18" s="44" t="n">
         <x:f>COUNTIFS('Lịch chi tiết'!$E$7:$E$256,$A18,'Lịch chi tiết'!$B$7:$B$256,3,'Lịch chi tiết'!$M$7:$M$256,"Done")</x:f>
@@ -16291,7 +16335,7 @@
       </x:c>
       <x:c r="G18" s="45" t="n">
         <x:f>SUM(B18:F18)</x:f>
-        <x:v>10</x:v>
+        <x:v>20</x:v>
       </x:c>
     </x:row>
     <x:row r="19" s="25" customFormat="1" ht="15" customHeight="1">
@@ -16306,7 +16350,7 @@
       </x:c>
       <x:c r="C19" s="44" t="n">
         <x:f>COUNTIFS('Lịch chi tiết'!$E$7:$E$256,$A19,'Lịch chi tiết'!$B$7:$B$256,2,'Lịch chi tiết'!$M$7:$M$256,"Done")</x:f>
-        <x:v>0</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D19" s="44" t="n">
         <x:f>COUNTIFS('Lịch chi tiết'!$E$7:$E$256,$A19,'Lịch chi tiết'!$B$7:$B$256,3,'Lịch chi tiết'!$M$7:$M$256,"Done")</x:f>
@@ -16322,7 +16366,7 @@
       </x:c>
       <x:c r="G19" s="45" t="n">
         <x:f>SUM(B19:F19)</x:f>
-        <x:v>10</x:v>
+        <x:v>20</x:v>
       </x:c>
     </x:row>
     <x:row r="20" s="25" customFormat="1" ht="15" customHeight="1">
@@ -16337,7 +16381,7 @@
       </x:c>
       <x:c r="C20" s="44" t="n">
         <x:f>COUNTIFS('Lịch chi tiết'!$E$7:$E$256,$A20,'Lịch chi tiết'!$B$7:$B$256,2,'Lịch chi tiết'!$M$7:$M$256,"Done")</x:f>
-        <x:v>0</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D20" s="44" t="n">
         <x:f>COUNTIFS('Lịch chi tiết'!$E$7:$E$256,$A20,'Lịch chi tiết'!$B$7:$B$256,3,'Lịch chi tiết'!$M$7:$M$256,"Done")</x:f>
@@ -16353,7 +16397,7 @@
       </x:c>
       <x:c r="G20" s="45" t="n">
         <x:f>SUM(B20:F20)</x:f>
-        <x:v>10</x:v>
+        <x:v>20</x:v>
       </x:c>
     </x:row>
     <x:row r="21" s="25" customFormat="1" ht="15" customHeight="1">
@@ -16368,7 +16412,7 @@
       </x:c>
       <x:c r="C21" s="45" t="n">
         <x:f>SUM(C16:C20)</x:f>
-        <x:v>0</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="D21" s="45" t="n">
         <x:f>SUM(D16:D20)</x:f>
@@ -16384,7 +16428,7 @@
       </x:c>
       <x:c r="G21" s="45" t="n">
         <x:f>SUM(G16:G20)</x:f>
-        <x:v>48</x:v>
+        <x:v>96</x:v>
       </x:c>
     </x:row>
     <x:row r="24" s="25" customFormat="1" ht="15" customHeight="1">
@@ -16443,7 +16487,7 @@
       </x:c>
       <x:c r="C26" s="47" t="n">
         <x:f>IF($B$2=0,0,C16/$B$2)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.8</x:v>
       </x:c>
       <x:c r="D26" s="47" t="n">
         <x:f>IF($B$2=0,0,D16/$B$2)</x:f>
@@ -16459,7 +16503,7 @@
       </x:c>
       <x:c r="G26" s="48" t="n">
         <x:f>IF($B$2=0,0,G16/($B$2*5))</x:f>
-        <x:v>0.2</x:v>
+        <x:v>0.36</x:v>
       </x:c>
     </x:row>
     <x:row r="27" s="25" customFormat="1" ht="15" customHeight="1">
@@ -16474,7 +16518,7 @@
       </x:c>
       <x:c r="C27" s="47" t="n">
         <x:f>IF($B$2=0,0,C17/$B$2)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D27" s="47" t="n">
         <x:f>IF($B$2=0,0,D17/$B$2)</x:f>
@@ -16490,7 +16534,7 @@
       </x:c>
       <x:c r="G27" s="48" t="n">
         <x:f>IF($B$2=0,0,G17/($B$2*5))</x:f>
-        <x:v>0.16</x:v>
+        <x:v>0.36</x:v>
       </x:c>
     </x:row>
     <x:row r="28" s="25" customFormat="1" ht="15" customHeight="1">
@@ -16505,7 +16549,7 @@
       </x:c>
       <x:c r="C28" s="47" t="n">
         <x:f>IF($B$2=0,0,C18/$B$2)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D28" s="47" t="n">
         <x:f>IF($B$2=0,0,D18/$B$2)</x:f>
@@ -16521,7 +16565,7 @@
       </x:c>
       <x:c r="G28" s="48" t="n">
         <x:f>IF($B$2=0,0,G18/($B$2*5))</x:f>
-        <x:v>0.2</x:v>
+        <x:v>0.4</x:v>
       </x:c>
     </x:row>
     <x:row r="29" s="25" customFormat="1" ht="15" customHeight="1">
@@ -16536,7 +16580,7 @@
       </x:c>
       <x:c r="C29" s="47" t="n">
         <x:f>IF($B$2=0,0,C19/$B$2)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D29" s="47" t="n">
         <x:f>IF($B$2=0,0,D19/$B$2)</x:f>
@@ -16552,7 +16596,7 @@
       </x:c>
       <x:c r="G29" s="48" t="n">
         <x:f>IF($B$2=0,0,G19/($B$2*5))</x:f>
-        <x:v>0.2</x:v>
+        <x:v>0.4</x:v>
       </x:c>
     </x:row>
     <x:row r="30" s="25" customFormat="1" ht="15" customHeight="1">
@@ -16567,7 +16611,7 @@
       </x:c>
       <x:c r="C30" s="47" t="n">
         <x:f>IF($B$2=0,0,C20/$B$2)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D30" s="47" t="n">
         <x:f>IF($B$2=0,0,D20/$B$2)</x:f>
@@ -16583,7 +16627,7 @@
       </x:c>
       <x:c r="G30" s="48" t="n">
         <x:f>IF($B$2=0,0,G20/($B$2*5))</x:f>
-        <x:v>0.2</x:v>
+        <x:v>0.4</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -16601,6 +16645,6 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb51e003be7bd41ab"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb42bc4e4d84640b4"/>
 </x:worksheet>
 </file>
</xml_diff>